<commit_message>
ActualizaciÃ³n completa del proyecto: mejoras en controladores, migraciones, seeders y componentes frontend
</commit_message>
<xml_diff>
--- a/backend/database/seeders/E2022bEstudiantesDatos.xlsx
+++ b/backend/database/seeders/E2022bEstudiantesDatos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\bebrascubarui\api\database\seeders\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\bebrascuba\api\database\seeders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE39C435-CF19-4CBB-91E2-5699A6B99372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF489ED-2DD1-4650-A9E5-1AC9C19FE6AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{A1482836-5B10-4DA2-BEF9-B536FE750C30}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A1482836-5B10-4DA2-BEF9-B536FE750C30}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$P$327</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -2448,11 +2457,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2460,7 +2469,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2468,13 +2477,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2482,7 +2491,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2490,7 +2499,7 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2865,17 +2874,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F9B48B8-4818-484F-9B88-D707BC38F446}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:P327"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.25" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.75" customWidth="1"/>
+    <col min="15" max="15" width="25.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2923,7 +2932,7 @@
       </c>
       <c r="P1" s="5"/>
     </row>
-    <row r="2" spans="1:16" hidden="1">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
@@ -2969,7 +2978,7 @@
       </c>
       <c r="P2" s="5"/>
     </row>
-    <row r="3" spans="1:16" hidden="1">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>15</v>
       </c>
@@ -3015,7 +3024,7 @@
       </c>
       <c r="P3" s="5"/>
     </row>
-    <row r="4" spans="1:16" hidden="1">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -3061,7 +3070,7 @@
       </c>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="1:16" hidden="1">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -3107,7 +3116,7 @@
       </c>
       <c r="P5" s="5"/>
     </row>
-    <row r="6" spans="1:16" hidden="1">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -3153,7 +3162,7 @@
       </c>
       <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="1:16" hidden="1">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>329</v>
       </c>
@@ -3199,7 +3208,7 @@
       </c>
       <c r="P7" s="5"/>
     </row>
-    <row r="8" spans="1:16" hidden="1">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
@@ -3245,7 +3254,7 @@
       </c>
       <c r="P8" s="5"/>
     </row>
-    <row r="9" spans="1:16" hidden="1">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>22</v>
       </c>
@@ -3291,7 +3300,7 @@
       </c>
       <c r="P9" s="5"/>
     </row>
-    <row r="10" spans="1:16" hidden="1">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
@@ -3337,7 +3346,7 @@
       </c>
       <c r="P10" s="5"/>
     </row>
-    <row r="11" spans="1:16" hidden="1">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>24</v>
       </c>
@@ -3383,7 +3392,7 @@
       </c>
       <c r="P11" s="5"/>
     </row>
-    <row r="12" spans="1:16" hidden="1">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>335</v>
       </c>
@@ -3429,7 +3438,7 @@
       </c>
       <c r="P12" s="5"/>
     </row>
-    <row r="13" spans="1:16" hidden="1">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>25</v>
       </c>
@@ -3475,7 +3484,7 @@
       </c>
       <c r="P13" s="5"/>
     </row>
-    <row r="14" spans="1:16" hidden="1">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>338</v>
       </c>
@@ -3521,7 +3530,7 @@
       </c>
       <c r="P14" s="5"/>
     </row>
-    <row r="15" spans="1:16" hidden="1">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>27</v>
       </c>
@@ -3567,7 +3576,7 @@
       </c>
       <c r="P15" s="5"/>
     </row>
-    <row r="16" spans="1:16" hidden="1">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
@@ -3613,7 +3622,7 @@
       </c>
       <c r="P16" s="5"/>
     </row>
-    <row r="17" spans="1:16" hidden="1">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>342</v>
       </c>
@@ -3659,7 +3668,7 @@
       </c>
       <c r="P17" s="5"/>
     </row>
-    <row r="18" spans="1:16" hidden="1">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>29</v>
       </c>
@@ -3705,7 +3714,7 @@
       </c>
       <c r="P18" s="5"/>
     </row>
-    <row r="19" spans="1:16" hidden="1">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>30</v>
       </c>
@@ -3751,7 +3760,7 @@
       </c>
       <c r="P19" s="5"/>
     </row>
-    <row r="20" spans="1:16" hidden="1">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>31</v>
       </c>
@@ -3797,7 +3806,7 @@
       </c>
       <c r="P20" s="5"/>
     </row>
-    <row r="21" spans="1:16" hidden="1">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>32</v>
       </c>
@@ -3843,7 +3852,7 @@
       </c>
       <c r="P21" s="5"/>
     </row>
-    <row r="22" spans="1:16" hidden="1">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>33</v>
       </c>
@@ -3889,7 +3898,7 @@
       </c>
       <c r="P22" s="5"/>
     </row>
-    <row r="23" spans="1:16" hidden="1">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>34</v>
       </c>
@@ -3935,7 +3944,7 @@
       </c>
       <c r="P23" s="5"/>
     </row>
-    <row r="24" spans="1:16" hidden="1">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>35</v>
       </c>
@@ -3981,7 +3990,7 @@
       </c>
       <c r="P24" s="5"/>
     </row>
-    <row r="25" spans="1:16" hidden="1">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>36</v>
       </c>
@@ -4027,7 +4036,7 @@
       </c>
       <c r="P25" s="5"/>
     </row>
-    <row r="26" spans="1:16" hidden="1">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>37</v>
       </c>
@@ -4073,7 +4082,7 @@
       </c>
       <c r="P26" s="5"/>
     </row>
-    <row r="27" spans="1:16" hidden="1">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>38</v>
       </c>
@@ -4119,7 +4128,7 @@
       </c>
       <c r="P27" s="5"/>
     </row>
-    <row r="28" spans="1:16" hidden="1">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>39</v>
       </c>
@@ -4165,7 +4174,7 @@
       </c>
       <c r="P28" s="5"/>
     </row>
-    <row r="29" spans="1:16" hidden="1">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>40</v>
       </c>
@@ -4211,7 +4220,7 @@
       </c>
       <c r="P29" s="5"/>
     </row>
-    <row r="30" spans="1:16" hidden="1">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>41</v>
       </c>
@@ -4257,7 +4266,7 @@
       </c>
       <c r="P30" s="5"/>
     </row>
-    <row r="31" spans="1:16" hidden="1">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>357</v>
       </c>
@@ -4303,7 +4312,7 @@
       </c>
       <c r="P31" s="5"/>
     </row>
-    <row r="32" spans="1:16" hidden="1">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>42</v>
       </c>
@@ -4349,7 +4358,7 @@
       </c>
       <c r="P32" s="5"/>
     </row>
-    <row r="33" spans="1:16" hidden="1">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>43</v>
       </c>
@@ -4395,7 +4404,7 @@
       </c>
       <c r="P33" s="5"/>
     </row>
-    <row r="34" spans="1:16" hidden="1">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>44</v>
       </c>
@@ -4441,7 +4450,7 @@
       </c>
       <c r="P34" s="5"/>
     </row>
-    <row r="35" spans="1:16" hidden="1">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>362</v>
       </c>
@@ -4487,7 +4496,7 @@
       </c>
       <c r="P35" s="5"/>
     </row>
-    <row r="36" spans="1:16" hidden="1">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>45</v>
       </c>
@@ -4533,7 +4542,7 @@
       </c>
       <c r="P36" s="5"/>
     </row>
-    <row r="37" spans="1:16" hidden="1">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>46</v>
       </c>
@@ -4579,7 +4588,7 @@
       </c>
       <c r="P37" s="5"/>
     </row>
-    <row r="38" spans="1:16" hidden="1">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>366</v>
       </c>
@@ -4625,7 +4634,7 @@
       </c>
       <c r="P38" s="5"/>
     </row>
-    <row r="39" spans="1:16" hidden="1">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>47</v>
       </c>
@@ -4671,7 +4680,7 @@
       </c>
       <c r="P39" s="5"/>
     </row>
-    <row r="40" spans="1:16" hidden="1">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>48</v>
       </c>
@@ -4717,7 +4726,7 @@
       </c>
       <c r="P40" s="5"/>
     </row>
-    <row r="41" spans="1:16" hidden="1">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>49</v>
       </c>
@@ -4763,7 +4772,7 @@
       </c>
       <c r="P41" s="5"/>
     </row>
-    <row r="42" spans="1:16" hidden="1">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>50</v>
       </c>
@@ -4809,7 +4818,7 @@
       </c>
       <c r="P42" s="5"/>
     </row>
-    <row r="43" spans="1:16" hidden="1">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>51</v>
       </c>
@@ -4855,7 +4864,7 @@
       </c>
       <c r="P43" s="5"/>
     </row>
-    <row r="44" spans="1:16" hidden="1">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>52</v>
       </c>
@@ -4901,7 +4910,7 @@
       </c>
       <c r="P44" s="5"/>
     </row>
-    <row r="45" spans="1:16" hidden="1">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>53</v>
       </c>
@@ -4947,7 +4956,7 @@
       </c>
       <c r="P45" s="5"/>
     </row>
-    <row r="46" spans="1:16" hidden="1">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>54</v>
       </c>
@@ -4993,7 +5002,7 @@
       </c>
       <c r="P46" s="5"/>
     </row>
-    <row r="47" spans="1:16" hidden="1">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>55</v>
       </c>
@@ -5039,7 +5048,7 @@
       </c>
       <c r="P47" s="5"/>
     </row>
-    <row r="48" spans="1:16" hidden="1">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
         <v>56</v>
       </c>
@@ -5085,7 +5094,7 @@
       </c>
       <c r="P48" s="5"/>
     </row>
-    <row r="49" spans="1:16" hidden="1">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
         <v>57</v>
       </c>
@@ -5131,7 +5140,7 @@
       </c>
       <c r="P49" s="5"/>
     </row>
-    <row r="50" spans="1:16" hidden="1">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>58</v>
       </c>
@@ -5177,7 +5186,7 @@
       </c>
       <c r="P50" s="5"/>
     </row>
-    <row r="51" spans="1:16" hidden="1">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>59</v>
       </c>
@@ -5223,7 +5232,7 @@
       </c>
       <c r="P51" s="5"/>
     </row>
-    <row r="52" spans="1:16" hidden="1">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>60</v>
       </c>
@@ -5269,7 +5278,7 @@
       </c>
       <c r="P52" s="5"/>
     </row>
-    <row r="53" spans="1:16" hidden="1">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>61</v>
       </c>
@@ -5315,7 +5324,7 @@
       </c>
       <c r="P53" s="5"/>
     </row>
-    <row r="54" spans="1:16" hidden="1">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
         <v>62</v>
       </c>
@@ -5361,7 +5370,7 @@
       </c>
       <c r="P54" s="5"/>
     </row>
-    <row r="55" spans="1:16" hidden="1">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
         <v>63</v>
       </c>
@@ -5407,7 +5416,7 @@
       </c>
       <c r="P55" s="5"/>
     </row>
-    <row r="56" spans="1:16" hidden="1">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
         <v>64</v>
       </c>
@@ -5453,7 +5462,7 @@
       </c>
       <c r="P56" s="5"/>
     </row>
-    <row r="57" spans="1:16" hidden="1">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
         <v>65</v>
       </c>
@@ -5499,7 +5508,7 @@
       </c>
       <c r="P57" s="5"/>
     </row>
-    <row r="58" spans="1:16" hidden="1">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
         <v>66</v>
       </c>
@@ -5543,7 +5552,7 @@
       </c>
       <c r="P58" s="5"/>
     </row>
-    <row r="59" spans="1:16" hidden="1">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" s="5" t="s">
         <v>69</v>
       </c>
@@ -5589,7 +5598,7 @@
       </c>
       <c r="P59" s="5"/>
     </row>
-    <row r="60" spans="1:16" hidden="1">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" s="5" t="s">
         <v>70</v>
       </c>
@@ -5635,7 +5644,7 @@
       </c>
       <c r="P60" s="5"/>
     </row>
-    <row r="61" spans="1:16" hidden="1">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" s="5" t="s">
         <v>71</v>
       </c>
@@ -5679,7 +5688,7 @@
       </c>
       <c r="P61" s="5"/>
     </row>
-    <row r="62" spans="1:16" hidden="1">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
         <v>392</v>
       </c>
@@ -5723,7 +5732,7 @@
       </c>
       <c r="P62" s="5"/>
     </row>
-    <row r="63" spans="1:16" hidden="1">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" s="5" t="s">
         <v>395</v>
       </c>
@@ -5769,7 +5778,7 @@
       </c>
       <c r="P63" s="5"/>
     </row>
-    <row r="64" spans="1:16" hidden="1">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
         <v>397</v>
       </c>
@@ -5815,7 +5824,7 @@
       </c>
       <c r="P64" s="5"/>
     </row>
-    <row r="65" spans="1:16" hidden="1">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
         <v>75</v>
       </c>
@@ -5861,7 +5870,7 @@
       </c>
       <c r="P65" s="5"/>
     </row>
-    <row r="66" spans="1:16" hidden="1">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
         <v>76</v>
       </c>
@@ -5907,7 +5916,7 @@
       </c>
       <c r="P66" s="5"/>
     </row>
-    <row r="67" spans="1:16" hidden="1">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
         <v>77</v>
       </c>
@@ -5953,7 +5962,7 @@
       </c>
       <c r="P67" s="5"/>
     </row>
-    <row r="68" spans="1:16" hidden="1">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
         <v>78</v>
       </c>
@@ -5999,7 +6008,7 @@
       </c>
       <c r="P68" s="5"/>
     </row>
-    <row r="69" spans="1:16" hidden="1">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
         <v>403</v>
       </c>
@@ -6045,7 +6054,7 @@
       </c>
       <c r="P69" s="5"/>
     </row>
-    <row r="70" spans="1:16" hidden="1">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
         <v>79</v>
       </c>
@@ -6091,7 +6100,7 @@
       </c>
       <c r="P70" s="5"/>
     </row>
-    <row r="71" spans="1:16" hidden="1">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A71" s="5" t="s">
         <v>80</v>
       </c>
@@ -6137,7 +6146,7 @@
       </c>
       <c r="P71" s="5"/>
     </row>
-    <row r="72" spans="1:16" hidden="1">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
         <v>81</v>
       </c>
@@ -6183,7 +6192,7 @@
       </c>
       <c r="P72" s="5"/>
     </row>
-    <row r="73" spans="1:16" hidden="1">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
         <v>82</v>
       </c>
@@ -6229,7 +6238,7 @@
       </c>
       <c r="P73" s="5"/>
     </row>
-    <row r="74" spans="1:16" hidden="1">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
         <v>83</v>
       </c>
@@ -6275,7 +6284,7 @@
       </c>
       <c r="P74" s="5"/>
     </row>
-    <row r="75" spans="1:16" hidden="1">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
         <v>84</v>
       </c>
@@ -6321,7 +6330,7 @@
       </c>
       <c r="P75" s="5"/>
     </row>
-    <row r="76" spans="1:16" hidden="1">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
         <v>85</v>
       </c>
@@ -6367,7 +6376,7 @@
       </c>
       <c r="P76" s="5"/>
     </row>
-    <row r="77" spans="1:16" hidden="1">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
         <v>86</v>
       </c>
@@ -6411,7 +6420,7 @@
       </c>
       <c r="P77" s="5"/>
     </row>
-    <row r="78" spans="1:16" hidden="1">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A78" s="5" t="s">
         <v>414</v>
       </c>
@@ -6455,7 +6464,7 @@
       </c>
       <c r="P78" s="5"/>
     </row>
-    <row r="79" spans="1:16" hidden="1">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
         <v>418</v>
       </c>
@@ -6499,7 +6508,7 @@
       </c>
       <c r="P79" s="5"/>
     </row>
-    <row r="80" spans="1:16" hidden="1">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
         <v>90</v>
       </c>
@@ -6543,7 +6552,7 @@
       </c>
       <c r="P80" s="5"/>
     </row>
-    <row r="81" spans="1:16" hidden="1">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
         <v>91</v>
       </c>
@@ -6587,7 +6596,7 @@
       </c>
       <c r="P81" s="5"/>
     </row>
-    <row r="82" spans="1:16" hidden="1">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
         <v>92</v>
       </c>
@@ -6631,7 +6640,7 @@
       </c>
       <c r="P82" s="5"/>
     </row>
-    <row r="83" spans="1:16" hidden="1">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
         <v>93</v>
       </c>
@@ -6675,7 +6684,7 @@
       </c>
       <c r="P83" s="5"/>
     </row>
-    <row r="84" spans="1:16" hidden="1">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
         <v>94</v>
       </c>
@@ -6719,7 +6728,7 @@
       </c>
       <c r="P84" s="5"/>
     </row>
-    <row r="85" spans="1:16" hidden="1">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
         <v>424</v>
       </c>
@@ -6763,7 +6772,7 @@
       </c>
       <c r="P85" s="5"/>
     </row>
-    <row r="86" spans="1:16" hidden="1">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
         <v>96</v>
       </c>
@@ -6811,7 +6820,7 @@
       </c>
       <c r="P86" s="5"/>
     </row>
-    <row r="87" spans="1:16" hidden="1">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
         <v>100</v>
       </c>
@@ -6855,7 +6864,7 @@
       </c>
       <c r="P87" s="5"/>
     </row>
-    <row r="88" spans="1:16" hidden="1">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A88" s="5" t="s">
         <v>104</v>
       </c>
@@ -6903,7 +6912,7 @@
       </c>
       <c r="P88" s="5"/>
     </row>
-    <row r="89" spans="1:16" hidden="1">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A89" s="5" t="s">
         <v>432</v>
       </c>
@@ -6951,7 +6960,7 @@
       </c>
       <c r="P89" s="5"/>
     </row>
-    <row r="90" spans="1:16" hidden="1">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
         <v>433</v>
       </c>
@@ -6995,7 +7004,7 @@
       </c>
       <c r="P90" s="5"/>
     </row>
-    <row r="91" spans="1:16" hidden="1">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A91" s="5" t="s">
         <v>107</v>
       </c>
@@ -7039,7 +7048,7 @@
       </c>
       <c r="P91" s="5"/>
     </row>
-    <row r="92" spans="1:16" hidden="1">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A92" s="5" t="s">
         <v>108</v>
       </c>
@@ -7083,7 +7092,7 @@
       </c>
       <c r="P92" s="5"/>
     </row>
-    <row r="93" spans="1:16" hidden="1">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A93" s="5" t="s">
         <v>109</v>
       </c>
@@ -7127,7 +7136,7 @@
       </c>
       <c r="P93" s="5"/>
     </row>
-    <row r="94" spans="1:16" hidden="1">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
         <v>689</v>
       </c>
@@ -7171,7 +7180,7 @@
       </c>
       <c r="P94" s="5"/>
     </row>
-    <row r="95" spans="1:16" hidden="1">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A95" s="5" t="s">
         <v>110</v>
       </c>
@@ -7215,7 +7224,7 @@
       </c>
       <c r="P95" s="5"/>
     </row>
-    <row r="96" spans="1:16" hidden="1">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A96" s="5" t="s">
         <v>111</v>
       </c>
@@ -7259,7 +7268,7 @@
       </c>
       <c r="P96" s="5"/>
     </row>
-    <row r="97" spans="1:16" hidden="1">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A97" s="5" t="s">
         <v>113</v>
       </c>
@@ -7305,7 +7314,7 @@
       </c>
       <c r="P97" s="5"/>
     </row>
-    <row r="98" spans="1:16" hidden="1">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A98" s="5" t="s">
         <v>117</v>
       </c>
@@ -7349,7 +7358,7 @@
       </c>
       <c r="P98" s="5"/>
     </row>
-    <row r="99" spans="1:16" hidden="1">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A99" s="5" t="s">
         <v>118</v>
       </c>
@@ -7393,7 +7402,7 @@
       </c>
       <c r="P99" s="5"/>
     </row>
-    <row r="100" spans="1:16" hidden="1">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A100" s="5" t="s">
         <v>450</v>
       </c>
@@ -7437,7 +7446,7 @@
       </c>
       <c r="P100" s="5"/>
     </row>
-    <row r="101" spans="1:16" hidden="1">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A101" s="5" t="s">
         <v>119</v>
       </c>
@@ -7481,7 +7490,7 @@
       </c>
       <c r="P101" s="5"/>
     </row>
-    <row r="102" spans="1:16" hidden="1">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
         <v>120</v>
       </c>
@@ -7525,7 +7534,7 @@
       </c>
       <c r="P102" s="5"/>
     </row>
-    <row r="103" spans="1:16" hidden="1">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A103" s="5" t="s">
         <v>456</v>
       </c>
@@ -7569,7 +7578,7 @@
       </c>
       <c r="P103" s="5"/>
     </row>
-    <row r="104" spans="1:16" hidden="1">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A104" s="5" t="s">
         <v>121</v>
       </c>
@@ -7613,7 +7622,7 @@
       </c>
       <c r="P104" s="5"/>
     </row>
-    <row r="105" spans="1:16" hidden="1">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A105" s="5" t="s">
         <v>122</v>
       </c>
@@ -7657,7 +7666,7 @@
       </c>
       <c r="P105" s="5"/>
     </row>
-    <row r="106" spans="1:16" hidden="1">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A106" s="5" t="s">
         <v>123</v>
       </c>
@@ -7701,7 +7710,7 @@
       </c>
       <c r="P106" s="5"/>
     </row>
-    <row r="107" spans="1:16" hidden="1">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A107" s="5" t="s">
         <v>124</v>
       </c>
@@ -7745,7 +7754,7 @@
       </c>
       <c r="P107" s="5"/>
     </row>
-    <row r="108" spans="1:16" hidden="1">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A108" s="5" t="s">
         <v>125</v>
       </c>
@@ -7791,7 +7800,7 @@
       </c>
       <c r="P108" s="5"/>
     </row>
-    <row r="109" spans="1:16" hidden="1">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A109" s="5" t="s">
         <v>465</v>
       </c>
@@ -7835,7 +7844,7 @@
       </c>
       <c r="P109" s="5"/>
     </row>
-    <row r="110" spans="1:16" hidden="1">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A110" s="5" t="s">
         <v>126</v>
       </c>
@@ -7879,7 +7888,7 @@
       </c>
       <c r="P110" s="5"/>
     </row>
-    <row r="111" spans="1:16" hidden="1">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A111" s="5" t="s">
         <v>127</v>
       </c>
@@ -7925,7 +7934,7 @@
       </c>
       <c r="P111" s="5"/>
     </row>
-    <row r="112" spans="1:16" hidden="1">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A112" s="5" t="s">
         <v>469</v>
       </c>
@@ -7969,7 +7978,7 @@
       </c>
       <c r="P112" s="5"/>
     </row>
-    <row r="113" spans="1:16" hidden="1">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A113" s="5" t="s">
         <v>128</v>
       </c>
@@ -8013,7 +8022,7 @@
       </c>
       <c r="P113" s="5"/>
     </row>
-    <row r="114" spans="1:16" hidden="1">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A114" s="5" t="s">
         <v>129</v>
       </c>
@@ -8057,7 +8066,7 @@
       </c>
       <c r="P114" s="5"/>
     </row>
-    <row r="115" spans="1:16" hidden="1">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A115" s="5" t="s">
         <v>473</v>
       </c>
@@ -8105,7 +8114,7 @@
       </c>
       <c r="P115" s="5"/>
     </row>
-    <row r="116" spans="1:16" hidden="1">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A116" s="5" t="s">
         <v>478</v>
       </c>
@@ -8153,7 +8162,7 @@
       </c>
       <c r="P116" s="5"/>
     </row>
-    <row r="117" spans="1:16" hidden="1">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A117" s="5" t="s">
         <v>131</v>
       </c>
@@ -8201,7 +8210,7 @@
       </c>
       <c r="P117" s="5"/>
     </row>
-    <row r="118" spans="1:16" hidden="1">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A118" s="5" t="s">
         <v>132</v>
       </c>
@@ -8249,7 +8258,7 @@
       </c>
       <c r="P118" s="5"/>
     </row>
-    <row r="119" spans="1:16" hidden="1">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A119" s="5" t="s">
         <v>483</v>
       </c>
@@ -8297,7 +8306,7 @@
       </c>
       <c r="P119" s="5"/>
     </row>
-    <row r="120" spans="1:16" hidden="1">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A120" s="5" t="s">
         <v>690</v>
       </c>
@@ -8345,7 +8354,7 @@
       </c>
       <c r="P120" s="5"/>
     </row>
-    <row r="121" spans="1:16" hidden="1">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A121" s="5" t="s">
         <v>133</v>
       </c>
@@ -8393,7 +8402,7 @@
       </c>
       <c r="P121" s="5"/>
     </row>
-    <row r="122" spans="1:16" hidden="1">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A122" s="5" t="s">
         <v>490</v>
       </c>
@@ -8441,7 +8450,7 @@
       </c>
       <c r="P122" s="5"/>
     </row>
-    <row r="123" spans="1:16" hidden="1">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A123" s="5" t="s">
         <v>134</v>
       </c>
@@ -8489,7 +8498,7 @@
       </c>
       <c r="P123" s="5"/>
     </row>
-    <row r="124" spans="1:16" hidden="1">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A124" s="5" t="s">
         <v>135</v>
       </c>
@@ -8537,7 +8546,7 @@
       </c>
       <c r="P124" s="5"/>
     </row>
-    <row r="125" spans="1:16" hidden="1">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A125" s="5" t="s">
         <v>136</v>
       </c>
@@ -8585,7 +8594,7 @@
       </c>
       <c r="P125" s="5"/>
     </row>
-    <row r="126" spans="1:16" hidden="1">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A126" s="5" t="s">
         <v>137</v>
       </c>
@@ -8633,7 +8642,7 @@
       </c>
       <c r="P126" s="5"/>
     </row>
-    <row r="127" spans="1:16" hidden="1">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A127" s="5" t="s">
         <v>138</v>
       </c>
@@ -8681,7 +8690,7 @@
       </c>
       <c r="P127" s="5"/>
     </row>
-    <row r="128" spans="1:16" hidden="1">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A128" s="5" t="s">
         <v>139</v>
       </c>
@@ -8729,7 +8738,7 @@
       </c>
       <c r="P128" s="5"/>
     </row>
-    <row r="129" spans="1:16" hidden="1">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A129" s="5" t="s">
         <v>498</v>
       </c>
@@ -8777,7 +8786,7 @@
       </c>
       <c r="P129" s="5"/>
     </row>
-    <row r="130" spans="1:16" hidden="1">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A130" s="5" t="s">
         <v>140</v>
       </c>
@@ -8825,7 +8834,7 @@
       </c>
       <c r="P130" s="5"/>
     </row>
-    <row r="131" spans="1:16" hidden="1">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A131" s="5" t="s">
         <v>141</v>
       </c>
@@ -8873,7 +8882,7 @@
       </c>
       <c r="P131" s="5"/>
     </row>
-    <row r="132" spans="1:16" hidden="1">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A132" s="5" t="s">
         <v>502</v>
       </c>
@@ -8921,7 +8930,7 @@
       </c>
       <c r="P132" s="5"/>
     </row>
-    <row r="133" spans="1:16" hidden="1">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A133" s="5" t="s">
         <v>142</v>
       </c>
@@ -8969,7 +8978,7 @@
       </c>
       <c r="P133" s="5"/>
     </row>
-    <row r="134" spans="1:16" hidden="1">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A134" s="5" t="s">
         <v>505</v>
       </c>
@@ -9017,7 +9026,7 @@
       </c>
       <c r="P134" s="5"/>
     </row>
-    <row r="135" spans="1:16" hidden="1">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A135" s="5" t="s">
         <v>143</v>
       </c>
@@ -9065,7 +9074,7 @@
       </c>
       <c r="P135" s="5"/>
     </row>
-    <row r="136" spans="1:16" hidden="1">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A136" s="5" t="s">
         <v>144</v>
       </c>
@@ -9113,7 +9122,7 @@
       </c>
       <c r="P136" s="5"/>
     </row>
-    <row r="137" spans="1:16">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A137" s="5" t="s">
         <v>145</v>
       </c>
@@ -9157,7 +9166,7 @@
       </c>
       <c r="P137" s="5"/>
     </row>
-    <row r="138" spans="1:16" hidden="1">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A138" s="5" t="s">
         <v>147</v>
       </c>
@@ -9205,7 +9214,7 @@
       </c>
       <c r="P138" s="5"/>
     </row>
-    <row r="139" spans="1:16" hidden="1">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A139" s="5" t="s">
         <v>148</v>
       </c>
@@ -9253,7 +9262,7 @@
       </c>
       <c r="P139" s="5"/>
     </row>
-    <row r="140" spans="1:16">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A140" s="5" t="s">
         <v>508</v>
       </c>
@@ -9297,7 +9306,7 @@
       </c>
       <c r="P140" s="5"/>
     </row>
-    <row r="141" spans="1:16" hidden="1">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A141" s="5" t="s">
         <v>149</v>
       </c>
@@ -9345,7 +9354,7 @@
       </c>
       <c r="P141" s="5"/>
     </row>
-    <row r="142" spans="1:16">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A142" s="5" t="s">
         <v>509</v>
       </c>
@@ -9389,7 +9398,7 @@
       </c>
       <c r="P142" s="5"/>
     </row>
-    <row r="143" spans="1:16">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A143" s="5" t="s">
         <v>512</v>
       </c>
@@ -9433,7 +9442,7 @@
       </c>
       <c r="P143" s="5"/>
     </row>
-    <row r="144" spans="1:16">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A144" s="5" t="s">
         <v>150</v>
       </c>
@@ -9477,7 +9486,7 @@
       </c>
       <c r="P144" s="5"/>
     </row>
-    <row r="145" spans="1:16">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A145" s="5" t="s">
         <v>151</v>
       </c>
@@ -9521,7 +9530,7 @@
       </c>
       <c r="P145" s="5"/>
     </row>
-    <row r="146" spans="1:16">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A146" s="5" t="s">
         <v>152</v>
       </c>
@@ -9565,7 +9574,7 @@
       </c>
       <c r="P146" s="5"/>
     </row>
-    <row r="147" spans="1:16">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A147" s="5" t="s">
         <v>153</v>
       </c>
@@ -9609,7 +9618,7 @@
       </c>
       <c r="P147" s="5"/>
     </row>
-    <row r="148" spans="1:16">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A148" s="5" t="s">
         <v>154</v>
       </c>
@@ -9653,7 +9662,7 @@
       </c>
       <c r="P148" s="5"/>
     </row>
-    <row r="149" spans="1:16">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A149" s="5" t="s">
         <v>522</v>
       </c>
@@ -9697,7 +9706,7 @@
       </c>
       <c r="P149" s="5"/>
     </row>
-    <row r="150" spans="1:16">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A150" s="5" t="s">
         <v>155</v>
       </c>
@@ -9741,7 +9750,7 @@
       </c>
       <c r="P150" s="5"/>
     </row>
-    <row r="151" spans="1:16">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A151" s="5" t="s">
         <v>525</v>
       </c>
@@ -9785,7 +9794,7 @@
       </c>
       <c r="P151" s="5"/>
     </row>
-    <row r="152" spans="1:16">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A152" s="5" t="s">
         <v>156</v>
       </c>
@@ -9829,7 +9838,7 @@
       </c>
       <c r="P152" s="5"/>
     </row>
-    <row r="153" spans="1:16">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A153" s="5" t="s">
         <v>527</v>
       </c>
@@ -9873,7 +9882,7 @@
       </c>
       <c r="P153" s="5"/>
     </row>
-    <row r="154" spans="1:16">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A154" s="5" t="s">
         <v>529</v>
       </c>
@@ -9917,7 +9926,7 @@
       </c>
       <c r="P154" s="5"/>
     </row>
-    <row r="155" spans="1:16">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A155" s="5" t="s">
         <v>157</v>
       </c>
@@ -9961,7 +9970,7 @@
       </c>
       <c r="P155" s="5"/>
     </row>
-    <row r="156" spans="1:16" hidden="1">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A156" s="5" t="s">
         <v>531</v>
       </c>
@@ -10005,7 +10014,7 @@
       </c>
       <c r="P156" s="5"/>
     </row>
-    <row r="157" spans="1:16">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A157" s="5" t="s">
         <v>533</v>
       </c>
@@ -10049,7 +10058,7 @@
       </c>
       <c r="P157" s="5"/>
     </row>
-    <row r="158" spans="1:16">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A158" s="5" t="s">
         <v>535</v>
       </c>
@@ -10093,7 +10102,7 @@
       </c>
       <c r="P158" s="5"/>
     </row>
-    <row r="159" spans="1:16">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A159" s="5" t="s">
         <v>160</v>
       </c>
@@ -10137,7 +10146,7 @@
       </c>
       <c r="P159" s="5"/>
     </row>
-    <row r="160" spans="1:16">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A160" s="5" t="s">
         <v>161</v>
       </c>
@@ -10181,7 +10190,7 @@
       </c>
       <c r="P160" s="5"/>
     </row>
-    <row r="161" spans="1:16" hidden="1">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A161" s="5" t="s">
         <v>162</v>
       </c>
@@ -10229,7 +10238,7 @@
       </c>
       <c r="P161" s="5"/>
     </row>
-    <row r="162" spans="1:16">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A162" s="5" t="s">
         <v>163</v>
       </c>
@@ -10273,7 +10282,7 @@
       </c>
       <c r="P162" s="5"/>
     </row>
-    <row r="163" spans="1:16">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A163" s="5" t="s">
         <v>164</v>
       </c>
@@ -10317,7 +10326,7 @@
       </c>
       <c r="P163" s="5"/>
     </row>
-    <row r="164" spans="1:16">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A164" s="5" t="s">
         <v>165</v>
       </c>
@@ -10361,7 +10370,7 @@
       </c>
       <c r="P164" s="5"/>
     </row>
-    <row r="165" spans="1:16" hidden="1">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A165" s="5" t="s">
         <v>540</v>
       </c>
@@ -10409,7 +10418,7 @@
       </c>
       <c r="P165" s="5"/>
     </row>
-    <row r="166" spans="1:16">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A166" s="5" t="s">
         <v>166</v>
       </c>
@@ -10453,7 +10462,7 @@
       </c>
       <c r="P166" s="5"/>
     </row>
-    <row r="167" spans="1:16">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A167" s="5" t="s">
         <v>541</v>
       </c>
@@ -10497,7 +10506,7 @@
       </c>
       <c r="P167" s="5"/>
     </row>
-    <row r="168" spans="1:16">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A168" s="5" t="s">
         <v>543</v>
       </c>
@@ -10541,7 +10550,7 @@
       </c>
       <c r="P168" s="5"/>
     </row>
-    <row r="169" spans="1:16">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A169" s="5" t="s">
         <v>167</v>
       </c>
@@ -10585,7 +10594,7 @@
       </c>
       <c r="P169" s="5"/>
     </row>
-    <row r="170" spans="1:16">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A170" s="5" t="s">
         <v>168</v>
       </c>
@@ -10629,7 +10638,7 @@
       </c>
       <c r="P170" s="5"/>
     </row>
-    <row r="171" spans="1:16">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A171" s="5" t="s">
         <v>169</v>
       </c>
@@ -10673,7 +10682,7 @@
       </c>
       <c r="P171" s="5"/>
     </row>
-    <row r="172" spans="1:16">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A172" s="5" t="s">
         <v>170</v>
       </c>
@@ -10717,7 +10726,7 @@
       </c>
       <c r="P172" s="5"/>
     </row>
-    <row r="173" spans="1:16">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A173" s="5" t="s">
         <v>548</v>
       </c>
@@ -10761,7 +10770,7 @@
       </c>
       <c r="P173" s="5"/>
     </row>
-    <row r="174" spans="1:16">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A174" s="5" t="s">
         <v>171</v>
       </c>
@@ -10805,7 +10814,7 @@
       </c>
       <c r="P174" s="5"/>
     </row>
-    <row r="175" spans="1:16">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A175" s="5" t="s">
         <v>551</v>
       </c>
@@ -10849,7 +10858,7 @@
       </c>
       <c r="P175" s="5"/>
     </row>
-    <row r="176" spans="1:16">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A176" s="5" t="s">
         <v>553</v>
       </c>
@@ -10893,7 +10902,7 @@
       </c>
       <c r="P176" s="5"/>
     </row>
-    <row r="177" spans="1:16">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A177" s="5" t="s">
         <v>172</v>
       </c>
@@ -10937,7 +10946,7 @@
       </c>
       <c r="P177" s="5"/>
     </row>
-    <row r="178" spans="1:16">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A178" s="5" t="s">
         <v>173</v>
       </c>
@@ -10981,7 +10990,7 @@
       </c>
       <c r="P178" s="5"/>
     </row>
-    <row r="179" spans="1:16" hidden="1">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A179" s="5" t="s">
         <v>557</v>
       </c>
@@ -11029,7 +11038,7 @@
       </c>
       <c r="P179" s="5"/>
     </row>
-    <row r="180" spans="1:16" hidden="1">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A180" s="5" t="s">
         <v>558</v>
       </c>
@@ -11077,7 +11086,7 @@
       </c>
       <c r="P180" s="5"/>
     </row>
-    <row r="181" spans="1:16">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A181" s="5" t="s">
         <v>174</v>
       </c>
@@ -11121,7 +11130,7 @@
       </c>
       <c r="P181" s="5"/>
     </row>
-    <row r="182" spans="1:16" hidden="1">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A182" s="5" t="s">
         <v>559</v>
       </c>
@@ -11169,7 +11178,7 @@
       </c>
       <c r="P182" s="5"/>
     </row>
-    <row r="183" spans="1:16" hidden="1">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A183" s="5" t="s">
         <v>175</v>
       </c>
@@ -11217,7 +11226,7 @@
       </c>
       <c r="P183" s="5"/>
     </row>
-    <row r="184" spans="1:16" hidden="1">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A184" s="5" t="s">
         <v>176</v>
       </c>
@@ -11265,7 +11274,7 @@
       </c>
       <c r="P184" s="5"/>
     </row>
-    <row r="185" spans="1:16" hidden="1">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A185" s="5" t="s">
         <v>560</v>
       </c>
@@ -11313,7 +11322,7 @@
       </c>
       <c r="P185" s="5"/>
     </row>
-    <row r="186" spans="1:16">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A186" s="5" t="s">
         <v>561</v>
       </c>
@@ -11357,7 +11366,7 @@
       </c>
       <c r="P186" s="5"/>
     </row>
-    <row r="187" spans="1:16">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A187" s="5" t="s">
         <v>177</v>
       </c>
@@ -11401,7 +11410,7 @@
       </c>
       <c r="P187" s="5"/>
     </row>
-    <row r="188" spans="1:16">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A188" s="5" t="s">
         <v>178</v>
       </c>
@@ -11445,7 +11454,7 @@
       </c>
       <c r="P188" s="5"/>
     </row>
-    <row r="189" spans="1:16">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A189" s="5" t="s">
         <v>179</v>
       </c>
@@ -11489,7 +11498,7 @@
       </c>
       <c r="P189" s="5"/>
     </row>
-    <row r="190" spans="1:16">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A190" s="5" t="s">
         <v>180</v>
       </c>
@@ -11533,7 +11542,7 @@
       </c>
       <c r="P190" s="5"/>
     </row>
-    <row r="191" spans="1:16">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A191" s="5" t="s">
         <v>567</v>
       </c>
@@ -11577,7 +11586,7 @@
       </c>
       <c r="P191" s="5"/>
     </row>
-    <row r="192" spans="1:16">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A192" s="5" t="s">
         <v>181</v>
       </c>
@@ -11621,7 +11630,7 @@
       </c>
       <c r="P192" s="5"/>
     </row>
-    <row r="193" spans="1:16">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A193" s="5" t="s">
         <v>570</v>
       </c>
@@ -11665,7 +11674,7 @@
       </c>
       <c r="P193" s="5"/>
     </row>
-    <row r="194" spans="1:16">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A194" s="5" t="s">
         <v>572</v>
       </c>
@@ -11709,7 +11718,7 @@
       </c>
       <c r="P194" s="5"/>
     </row>
-    <row r="195" spans="1:16">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A195" s="5" t="s">
         <v>182</v>
       </c>
@@ -11753,7 +11762,7 @@
       </c>
       <c r="P195" s="5"/>
     </row>
-    <row r="196" spans="1:16">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A196" s="5" t="s">
         <v>575</v>
       </c>
@@ -11797,7 +11806,7 @@
       </c>
       <c r="P196" s="5"/>
     </row>
-    <row r="197" spans="1:16">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A197" s="5" t="s">
         <v>183</v>
       </c>
@@ -11841,7 +11850,7 @@
       </c>
       <c r="P197" s="5"/>
     </row>
-    <row r="198" spans="1:16">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A198" s="5" t="s">
         <v>184</v>
       </c>
@@ -11885,7 +11894,7 @@
       </c>
       <c r="P198" s="5"/>
     </row>
-    <row r="199" spans="1:16">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A199" s="5" t="s">
         <v>185</v>
       </c>
@@ -11929,7 +11938,7 @@
       </c>
       <c r="P199" s="5"/>
     </row>
-    <row r="200" spans="1:16" hidden="1">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A200" s="5" t="s">
         <v>186</v>
       </c>
@@ -11973,7 +11982,7 @@
       </c>
       <c r="P200" s="5"/>
     </row>
-    <row r="201" spans="1:16" hidden="1">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A201" s="5" t="s">
         <v>581</v>
       </c>
@@ -12017,7 +12026,7 @@
       </c>
       <c r="P201" s="5"/>
     </row>
-    <row r="202" spans="1:16" hidden="1">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A202" s="5" t="s">
         <v>189</v>
       </c>
@@ -12061,7 +12070,7 @@
       </c>
       <c r="P202" s="5"/>
     </row>
-    <row r="203" spans="1:16" hidden="1">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A203" s="5" t="s">
         <v>691</v>
       </c>
@@ -12103,7 +12112,7 @@
       </c>
       <c r="P203" s="5"/>
     </row>
-    <row r="204" spans="1:16" hidden="1">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A204" s="5" t="s">
         <v>190</v>
       </c>
@@ -12147,7 +12156,7 @@
       </c>
       <c r="P204" s="5"/>
     </row>
-    <row r="205" spans="1:16" hidden="1">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A205" s="5" t="s">
         <v>191</v>
       </c>
@@ -12191,7 +12200,7 @@
       </c>
       <c r="P205" s="5"/>
     </row>
-    <row r="206" spans="1:16" hidden="1">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A206" s="5" t="s">
         <v>192</v>
       </c>
@@ -12235,7 +12244,7 @@
       </c>
       <c r="P206" s="5"/>
     </row>
-    <row r="207" spans="1:16" hidden="1">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A207" s="5" t="s">
         <v>193</v>
       </c>
@@ -12279,7 +12288,7 @@
       </c>
       <c r="P207" s="5"/>
     </row>
-    <row r="208" spans="1:16" hidden="1">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A208" s="5" t="s">
         <v>194</v>
       </c>
@@ -12323,7 +12332,7 @@
       </c>
       <c r="P208" s="5"/>
     </row>
-    <row r="209" spans="1:16" hidden="1">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A209" s="5" t="s">
         <v>197</v>
       </c>
@@ -12367,7 +12376,7 @@
       </c>
       <c r="P209" s="5"/>
     </row>
-    <row r="210" spans="1:16" hidden="1">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A210" s="5" t="s">
         <v>198</v>
       </c>
@@ -12411,7 +12420,7 @@
       </c>
       <c r="P210" s="5"/>
     </row>
-    <row r="211" spans="1:16" hidden="1">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A211" s="5" t="s">
         <v>201</v>
       </c>
@@ -12455,7 +12464,7 @@
       </c>
       <c r="P211" s="5"/>
     </row>
-    <row r="212" spans="1:16" hidden="1">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A212" s="5" t="s">
         <v>591</v>
       </c>
@@ -12499,7 +12508,7 @@
       </c>
       <c r="P212" s="5"/>
     </row>
-    <row r="213" spans="1:16" hidden="1">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A213" s="5" t="s">
         <v>202</v>
       </c>
@@ -12547,7 +12556,7 @@
       </c>
       <c r="P213" s="5"/>
     </row>
-    <row r="214" spans="1:16" hidden="1">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A214" s="5" t="s">
         <v>204</v>
       </c>
@@ -12595,7 +12604,7 @@
       </c>
       <c r="P214" s="5"/>
     </row>
-    <row r="215" spans="1:16" hidden="1">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A215" s="5" t="s">
         <v>205</v>
       </c>
@@ -12639,7 +12648,7 @@
       </c>
       <c r="P215" s="5"/>
     </row>
-    <row r="216" spans="1:16">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A216" s="5" t="s">
         <v>207</v>
       </c>
@@ -12683,7 +12692,7 @@
       </c>
       <c r="P216" s="5"/>
     </row>
-    <row r="217" spans="1:16" hidden="1">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A217" s="5" t="s">
         <v>208</v>
       </c>
@@ -12727,7 +12736,7 @@
       </c>
       <c r="P217" s="5"/>
     </row>
-    <row r="218" spans="1:16" hidden="1">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A218" s="5" t="s">
         <v>594</v>
       </c>
@@ -12775,7 +12784,7 @@
       </c>
       <c r="P218" s="5"/>
     </row>
-    <row r="219" spans="1:16" hidden="1">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A219" s="5" t="s">
         <v>597</v>
       </c>
@@ -12823,7 +12832,7 @@
       </c>
       <c r="P219" s="5"/>
     </row>
-    <row r="220" spans="1:16" hidden="1">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A220" s="5" t="s">
         <v>599</v>
       </c>
@@ -12871,7 +12880,7 @@
       </c>
       <c r="P220" s="5"/>
     </row>
-    <row r="221" spans="1:16" hidden="1">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A221" s="5" t="s">
         <v>209</v>
       </c>
@@ -12919,7 +12928,7 @@
       </c>
       <c r="P221" s="5"/>
     </row>
-    <row r="222" spans="1:16" hidden="1">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A222" s="5" t="s">
         <v>210</v>
       </c>
@@ -12967,7 +12976,7 @@
       </c>
       <c r="P222" s="5"/>
     </row>
-    <row r="223" spans="1:16" hidden="1">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A223" s="5" t="s">
         <v>211</v>
       </c>
@@ -13011,7 +13020,7 @@
       </c>
       <c r="P223" s="5"/>
     </row>
-    <row r="224" spans="1:16" hidden="1">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A224" s="5" t="s">
         <v>212</v>
       </c>
@@ -13059,7 +13068,7 @@
       </c>
       <c r="P224" s="5"/>
     </row>
-    <row r="225" spans="1:16" hidden="1">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A225" s="5" t="s">
         <v>603</v>
       </c>
@@ -13107,7 +13116,7 @@
       </c>
       <c r="P225" s="5"/>
     </row>
-    <row r="226" spans="1:16" hidden="1">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A226" s="5" t="s">
         <v>213</v>
       </c>
@@ -13155,7 +13164,7 @@
       </c>
       <c r="P226" s="5"/>
     </row>
-    <row r="227" spans="1:16" hidden="1">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A227" s="5" t="s">
         <v>606</v>
       </c>
@@ -13203,7 +13212,7 @@
       </c>
       <c r="P227" s="5"/>
     </row>
-    <row r="228" spans="1:16" hidden="1">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A228" s="5" t="s">
         <v>214</v>
       </c>
@@ -13251,7 +13260,7 @@
       </c>
       <c r="P228" s="5"/>
     </row>
-    <row r="229" spans="1:16" hidden="1">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A229" s="5" t="s">
         <v>215</v>
       </c>
@@ -13299,7 +13308,7 @@
       </c>
       <c r="P229" s="5"/>
     </row>
-    <row r="230" spans="1:16" hidden="1">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A230" s="5" t="s">
         <v>216</v>
       </c>
@@ -13347,7 +13356,7 @@
       </c>
       <c r="P230" s="5"/>
     </row>
-    <row r="231" spans="1:16" hidden="1">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A231" s="5" t="s">
         <v>611</v>
       </c>
@@ -13395,7 +13404,7 @@
       </c>
       <c r="P231" s="5"/>
     </row>
-    <row r="232" spans="1:16">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A232" s="5" t="s">
         <v>217</v>
       </c>
@@ -13439,7 +13448,7 @@
       </c>
       <c r="P232" s="5"/>
     </row>
-    <row r="233" spans="1:16" hidden="1">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A233" s="5" t="s">
         <v>218</v>
       </c>
@@ -13483,7 +13492,7 @@
       </c>
       <c r="P233" s="5"/>
     </row>
-    <row r="234" spans="1:16" hidden="1">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A234" s="5" t="s">
         <v>220</v>
       </c>
@@ -13527,7 +13536,7 @@
       </c>
       <c r="P234" s="5"/>
     </row>
-    <row r="235" spans="1:16">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A235" s="5" t="s">
         <v>221</v>
       </c>
@@ -13571,7 +13580,7 @@
       </c>
       <c r="P235" s="5"/>
     </row>
-    <row r="236" spans="1:16" hidden="1">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A236" s="5" t="s">
         <v>222</v>
       </c>
@@ -13619,7 +13628,7 @@
       </c>
       <c r="P236" s="5"/>
     </row>
-    <row r="237" spans="1:16" hidden="1">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A237" s="5" t="s">
         <v>223</v>
       </c>
@@ -13667,7 +13676,7 @@
       </c>
       <c r="P237" s="5"/>
     </row>
-    <row r="238" spans="1:16" hidden="1">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A238" s="5" t="s">
         <v>224</v>
       </c>
@@ -13715,7 +13724,7 @@
       </c>
       <c r="P238" s="5"/>
     </row>
-    <row r="239" spans="1:16" hidden="1">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A239" s="5" t="s">
         <v>225</v>
       </c>
@@ -13763,7 +13772,7 @@
       </c>
       <c r="P239" s="5"/>
     </row>
-    <row r="240" spans="1:16" hidden="1">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A240" s="5" t="s">
         <v>619</v>
       </c>
@@ -13811,7 +13820,7 @@
       </c>
       <c r="P240" s="5"/>
     </row>
-    <row r="241" spans="1:16" hidden="1">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A241" s="5" t="s">
         <v>226</v>
       </c>
@@ -13859,7 +13868,7 @@
       </c>
       <c r="P241" s="5"/>
     </row>
-    <row r="242" spans="1:16" hidden="1">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A242" s="5" t="s">
         <v>227</v>
       </c>
@@ -13907,7 +13916,7 @@
       </c>
       <c r="P242" s="5"/>
     </row>
-    <row r="243" spans="1:16" hidden="1">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A243" s="5" t="s">
         <v>228</v>
       </c>
@@ -13955,7 +13964,7 @@
       </c>
       <c r="P243" s="5"/>
     </row>
-    <row r="244" spans="1:16" hidden="1">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A244" s="5" t="s">
         <v>229</v>
       </c>
@@ -14003,7 +14012,7 @@
       </c>
       <c r="P244" s="5"/>
     </row>
-    <row r="245" spans="1:16" hidden="1">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A245" s="5" t="s">
         <v>230</v>
       </c>
@@ -14051,7 +14060,7 @@
       </c>
       <c r="P245" s="5"/>
     </row>
-    <row r="246" spans="1:16" hidden="1">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A246" s="5" t="s">
         <v>231</v>
       </c>
@@ -14099,7 +14108,7 @@
       </c>
       <c r="P246" s="5"/>
     </row>
-    <row r="247" spans="1:16" hidden="1">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A247" s="5" t="s">
         <v>232</v>
       </c>
@@ -14147,7 +14156,7 @@
       </c>
       <c r="P247" s="5"/>
     </row>
-    <row r="248" spans="1:16" hidden="1">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A248" s="5" t="s">
         <v>233</v>
       </c>
@@ -14195,7 +14204,7 @@
       </c>
       <c r="P248" s="5"/>
     </row>
-    <row r="249" spans="1:16" hidden="1">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A249" s="5" t="s">
         <v>234</v>
       </c>
@@ -14239,7 +14248,7 @@
       </c>
       <c r="P249" s="5"/>
     </row>
-    <row r="250" spans="1:16" hidden="1">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A250" s="5" t="s">
         <v>625</v>
       </c>
@@ -14287,7 +14296,7 @@
       </c>
       <c r="P250" s="5"/>
     </row>
-    <row r="251" spans="1:16">
+    <row r="251" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A251" s="5" t="s">
         <v>235</v>
       </c>
@@ -14331,7 +14340,7 @@
       </c>
       <c r="P251" s="5"/>
     </row>
-    <row r="252" spans="1:16">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A252" s="5" t="s">
         <v>236</v>
       </c>
@@ -14375,7 +14384,7 @@
       </c>
       <c r="P252" s="5"/>
     </row>
-    <row r="253" spans="1:16" hidden="1">
+    <row r="253" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A253" s="5" t="s">
         <v>626</v>
       </c>
@@ -14423,7 +14432,7 @@
       </c>
       <c r="P253" s="5"/>
     </row>
-    <row r="254" spans="1:16" hidden="1">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A254" s="5" t="s">
         <v>237</v>
       </c>
@@ -14471,7 +14480,7 @@
       </c>
       <c r="P254" s="5"/>
     </row>
-    <row r="255" spans="1:16" hidden="1">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A255" s="5" t="s">
         <v>238</v>
       </c>
@@ -14515,7 +14524,7 @@
       </c>
       <c r="P255" s="5"/>
     </row>
-    <row r="256" spans="1:16" hidden="1">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A256" s="5" t="s">
         <v>631</v>
       </c>
@@ -14559,7 +14568,7 @@
       </c>
       <c r="P256" s="5"/>
     </row>
-    <row r="257" spans="1:16" hidden="1">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A257" s="5" t="s">
         <v>634</v>
       </c>
@@ -14607,7 +14616,7 @@
       </c>
       <c r="P257" s="5"/>
     </row>
-    <row r="258" spans="1:16" hidden="1">
+    <row r="258" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A258" s="5" t="s">
         <v>240</v>
       </c>
@@ -14655,7 +14664,7 @@
       </c>
       <c r="P258" s="5"/>
     </row>
-    <row r="259" spans="1:16" hidden="1">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A259" s="5" t="s">
         <v>636</v>
       </c>
@@ -14703,7 +14712,7 @@
       </c>
       <c r="P259" s="5"/>
     </row>
-    <row r="260" spans="1:16" hidden="1">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A260" s="5" t="s">
         <v>241</v>
       </c>
@@ -14751,7 +14760,7 @@
       </c>
       <c r="P260" s="5"/>
     </row>
-    <row r="261" spans="1:16" hidden="1">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A261" s="5" t="s">
         <v>639</v>
       </c>
@@ -14795,7 +14804,7 @@
       </c>
       <c r="P261" s="5"/>
     </row>
-    <row r="262" spans="1:16">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A262" s="5" t="s">
         <v>242</v>
       </c>
@@ -14839,7 +14848,7 @@
       </c>
       <c r="P262" s="5"/>
     </row>
-    <row r="263" spans="1:16" hidden="1">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A263" s="5" t="s">
         <v>640</v>
       </c>
@@ -14883,7 +14892,7 @@
       </c>
       <c r="P263" s="5"/>
     </row>
-    <row r="264" spans="1:16" hidden="1">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A264" s="5" t="s">
         <v>643</v>
       </c>
@@ -14931,7 +14940,7 @@
       </c>
       <c r="P264" s="5"/>
     </row>
-    <row r="265" spans="1:16" hidden="1">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A265" s="5" t="s">
         <v>243</v>
       </c>
@@ -14975,7 +14984,7 @@
       </c>
       <c r="P265" s="5"/>
     </row>
-    <row r="266" spans="1:16" hidden="1">
+    <row r="266" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A266" s="5" t="s">
         <v>244</v>
       </c>
@@ -15023,7 +15032,7 @@
       </c>
       <c r="P266" s="5"/>
     </row>
-    <row r="267" spans="1:16" hidden="1">
+    <row r="267" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A267" s="5" t="s">
         <v>245</v>
       </c>
@@ -15067,7 +15076,7 @@
       </c>
       <c r="P267" s="5"/>
     </row>
-    <row r="268" spans="1:16">
+    <row r="268" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A268" s="5" t="s">
         <v>248</v>
       </c>
@@ -15111,7 +15120,7 @@
       </c>
       <c r="P268" s="5"/>
     </row>
-    <row r="269" spans="1:16" hidden="1">
+    <row r="269" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A269" s="5" t="s">
         <v>249</v>
       </c>
@@ -15159,7 +15168,7 @@
       </c>
       <c r="P269" s="5"/>
     </row>
-    <row r="270" spans="1:16" hidden="1">
+    <row r="270" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A270" s="5" t="s">
         <v>647</v>
       </c>
@@ -15203,7 +15212,7 @@
       </c>
       <c r="P270" s="5"/>
     </row>
-    <row r="271" spans="1:16" hidden="1">
+    <row r="271" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A271" s="5" t="s">
         <v>250</v>
       </c>
@@ -15247,7 +15256,7 @@
       </c>
       <c r="P271" s="5"/>
     </row>
-    <row r="272" spans="1:16" hidden="1">
+    <row r="272" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A272" s="5" t="s">
         <v>654</v>
       </c>
@@ -15291,7 +15300,7 @@
       </c>
       <c r="P272" s="5"/>
     </row>
-    <row r="273" spans="1:16" hidden="1">
+    <row r="273" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A273" s="5" t="s">
         <v>251</v>
       </c>
@@ -15335,7 +15344,7 @@
       </c>
       <c r="P273" s="5"/>
     </row>
-    <row r="274" spans="1:16">
+    <row r="274" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A274" s="5" t="s">
         <v>252</v>
       </c>
@@ -15379,7 +15388,7 @@
       </c>
       <c r="P274" s="5"/>
     </row>
-    <row r="275" spans="1:16" hidden="1">
+    <row r="275" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A275" s="5" t="s">
         <v>253</v>
       </c>
@@ -15423,7 +15432,7 @@
       </c>
       <c r="P275" s="5"/>
     </row>
-    <row r="276" spans="1:16" hidden="1">
+    <row r="276" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A276" s="5" t="s">
         <v>255</v>
       </c>
@@ -15467,7 +15476,7 @@
       </c>
       <c r="P276" s="5"/>
     </row>
-    <row r="277" spans="1:16" hidden="1">
+    <row r="277" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A277" s="5" t="s">
         <v>256</v>
       </c>
@@ -15511,7 +15520,7 @@
       </c>
       <c r="P277" s="5"/>
     </row>
-    <row r="278" spans="1:16">
+    <row r="278" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A278" s="5" t="s">
         <v>257</v>
       </c>
@@ -15555,7 +15564,7 @@
       </c>
       <c r="P278" s="5"/>
     </row>
-    <row r="279" spans="1:16" hidden="1">
+    <row r="279" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A279" s="5" t="s">
         <v>258</v>
       </c>
@@ -15599,7 +15608,7 @@
       </c>
       <c r="P279" s="5"/>
     </row>
-    <row r="280" spans="1:16" hidden="1">
+    <row r="280" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A280" s="5" t="s">
         <v>259</v>
       </c>
@@ -15643,7 +15652,7 @@
       </c>
       <c r="P280" s="5"/>
     </row>
-    <row r="281" spans="1:16" hidden="1">
+    <row r="281" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A281" s="5" t="s">
         <v>260</v>
       </c>
@@ -15687,7 +15696,7 @@
       </c>
       <c r="P281" s="5"/>
     </row>
-    <row r="282" spans="1:16" hidden="1">
+    <row r="282" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A282" s="5" t="s">
         <v>261</v>
       </c>
@@ -15731,7 +15740,7 @@
       </c>
       <c r="P282" s="5"/>
     </row>
-    <row r="283" spans="1:16" hidden="1">
+    <row r="283" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A283" s="5" t="s">
         <v>262</v>
       </c>
@@ -15775,7 +15784,7 @@
       </c>
       <c r="P283" s="5"/>
     </row>
-    <row r="284" spans="1:16" hidden="1">
+    <row r="284" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A284" s="5" t="s">
         <v>263</v>
       </c>
@@ -15819,7 +15828,7 @@
       </c>
       <c r="P284" s="5"/>
     </row>
-    <row r="285" spans="1:16" hidden="1">
+    <row r="285" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A285" s="5" t="s">
         <v>264</v>
       </c>
@@ -15863,7 +15872,7 @@
       </c>
       <c r="P285" s="5"/>
     </row>
-    <row r="286" spans="1:16" hidden="1">
+    <row r="286" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A286" s="5" t="s">
         <v>265</v>
       </c>
@@ -15907,7 +15916,7 @@
       </c>
       <c r="P286" s="5"/>
     </row>
-    <row r="287" spans="1:16" hidden="1">
+    <row r="287" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A287" s="5" t="s">
         <v>266</v>
       </c>
@@ -15951,7 +15960,7 @@
       </c>
       <c r="P287" s="5"/>
     </row>
-    <row r="288" spans="1:16" hidden="1">
+    <row r="288" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A288" s="5" t="s">
         <v>267</v>
       </c>
@@ -15995,7 +16004,7 @@
       </c>
       <c r="P288" s="5"/>
     </row>
-    <row r="289" spans="1:16" hidden="1">
+    <row r="289" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A289" s="5" t="s">
         <v>268</v>
       </c>
@@ -16039,7 +16048,7 @@
       </c>
       <c r="P289" s="5"/>
     </row>
-    <row r="290" spans="1:16" hidden="1">
+    <row r="290" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A290" s="5" t="s">
         <v>269</v>
       </c>
@@ -16083,7 +16092,7 @@
       </c>
       <c r="P290" s="5"/>
     </row>
-    <row r="291" spans="1:16" hidden="1">
+    <row r="291" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A291" s="5" t="s">
         <v>270</v>
       </c>
@@ -16127,7 +16136,7 @@
       </c>
       <c r="P291" s="5"/>
     </row>
-    <row r="292" spans="1:16" hidden="1">
+    <row r="292" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A292" s="5" t="s">
         <v>693</v>
       </c>
@@ -16171,7 +16180,7 @@
       </c>
       <c r="P292" s="5"/>
     </row>
-    <row r="293" spans="1:16" hidden="1">
+    <row r="293" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A293" s="5" t="s">
         <v>271</v>
       </c>
@@ -16215,7 +16224,7 @@
       </c>
       <c r="P293" s="5"/>
     </row>
-    <row r="294" spans="1:16" hidden="1">
+    <row r="294" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A294" s="5" t="s">
         <v>272</v>
       </c>
@@ -16257,7 +16266,7 @@
       </c>
       <c r="P294" s="5"/>
     </row>
-    <row r="295" spans="1:16">
+    <row r="295" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A295" s="5" t="s">
         <v>273</v>
       </c>
@@ -16301,7 +16310,7 @@
       </c>
       <c r="P295" s="5"/>
     </row>
-    <row r="296" spans="1:16">
+    <row r="296" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A296" s="5" t="s">
         <v>274</v>
       </c>
@@ -16345,7 +16354,7 @@
       </c>
       <c r="P296" s="5"/>
     </row>
-    <row r="297" spans="1:16" hidden="1">
+    <row r="297" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A297" s="5" t="s">
         <v>275</v>
       </c>
@@ -16389,7 +16398,7 @@
       </c>
       <c r="P297" s="5"/>
     </row>
-    <row r="298" spans="1:16" hidden="1">
+    <row r="298" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A298" s="5" t="s">
         <v>276</v>
       </c>
@@ -16433,7 +16442,7 @@
       </c>
       <c r="P298" s="5"/>
     </row>
-    <row r="299" spans="1:16" hidden="1">
+    <row r="299" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A299" s="5" t="s">
         <v>277</v>
       </c>
@@ -16477,7 +16486,7 @@
       </c>
       <c r="P299" s="5"/>
     </row>
-    <row r="300" spans="1:16" hidden="1">
+    <row r="300" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A300" s="5" t="s">
         <v>278</v>
       </c>
@@ -16521,7 +16530,7 @@
       </c>
       <c r="P300" s="5"/>
     </row>
-    <row r="301" spans="1:16" hidden="1">
+    <row r="301" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A301" s="5" t="s">
         <v>279</v>
       </c>
@@ -16565,7 +16574,7 @@
       </c>
       <c r="P301" s="5"/>
     </row>
-    <row r="302" spans="1:16" hidden="1">
+    <row r="302" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A302" s="5" t="s">
         <v>280</v>
       </c>
@@ -16609,7 +16618,7 @@
       </c>
       <c r="P302" s="5"/>
     </row>
-    <row r="303" spans="1:16" hidden="1">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A303" s="5" t="s">
         <v>281</v>
       </c>
@@ -16653,7 +16662,7 @@
       </c>
       <c r="P303" s="5"/>
     </row>
-    <row r="304" spans="1:16" hidden="1">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A304" s="5" t="s">
         <v>282</v>
       </c>
@@ -16697,7 +16706,7 @@
       </c>
       <c r="P304" s="5"/>
     </row>
-    <row r="305" spans="1:16" hidden="1">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A305" s="5" t="s">
         <v>676</v>
       </c>
@@ -16741,7 +16750,7 @@
       </c>
       <c r="P305" s="5"/>
     </row>
-    <row r="306" spans="1:16" hidden="1">
+    <row r="306" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A306" s="5" t="s">
         <v>677</v>
       </c>
@@ -16789,7 +16798,7 @@
       </c>
       <c r="P306" s="5"/>
     </row>
-    <row r="307" spans="1:16" hidden="1">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A307" s="5" t="s">
         <v>283</v>
       </c>
@@ -16833,7 +16842,7 @@
       </c>
       <c r="P307" s="5"/>
     </row>
-    <row r="308" spans="1:16" hidden="1">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A308" s="5" t="s">
         <v>284</v>
       </c>
@@ -16881,7 +16890,7 @@
       </c>
       <c r="P308" s="5"/>
     </row>
-    <row r="309" spans="1:16" hidden="1">
+    <row r="309" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A309" s="5" t="s">
         <v>678</v>
       </c>
@@ -16925,7 +16934,7 @@
       </c>
       <c r="P309" s="5"/>
     </row>
-    <row r="310" spans="1:16">
+    <row r="310" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A310" s="5" t="s">
         <v>679</v>
       </c>
@@ -16969,7 +16978,7 @@
       </c>
       <c r="P310" s="5"/>
     </row>
-    <row r="311" spans="1:16">
+    <row r="311" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A311" s="5" t="s">
         <v>285</v>
       </c>
@@ -17013,7 +17022,7 @@
       </c>
       <c r="P311" s="5"/>
     </row>
-    <row r="312" spans="1:16">
+    <row r="312" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A312" s="5" t="s">
         <v>286</v>
       </c>
@@ -17057,7 +17066,7 @@
       </c>
       <c r="P312" s="5"/>
     </row>
-    <row r="313" spans="1:16" hidden="1">
+    <row r="313" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A313" s="5" t="s">
         <v>287</v>
       </c>
@@ -17101,7 +17110,7 @@
       </c>
       <c r="P313" s="5"/>
     </row>
-    <row r="314" spans="1:16" hidden="1">
+    <row r="314" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A314" s="5" t="s">
         <v>290</v>
       </c>
@@ -17145,7 +17154,7 @@
       </c>
       <c r="P314" s="5"/>
     </row>
-    <row r="315" spans="1:16" hidden="1">
+    <row r="315" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A315" s="5" t="s">
         <v>291</v>
       </c>
@@ -17189,7 +17198,7 @@
       </c>
       <c r="P315" s="5"/>
     </row>
-    <row r="316" spans="1:16" hidden="1">
+    <row r="316" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A316" s="5" t="s">
         <v>684</v>
       </c>
@@ -17231,7 +17240,7 @@
       </c>
       <c r="P316" s="5"/>
     </row>
-    <row r="317" spans="1:16">
+    <row r="317" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A317" s="5" t="s">
         <v>295</v>
       </c>
@@ -17273,7 +17282,7 @@
       </c>
       <c r="P317" s="5"/>
     </row>
-    <row r="318" spans="1:16">
+    <row r="318" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A318" s="5" t="s">
         <v>296</v>
       </c>
@@ -17315,7 +17324,7 @@
       </c>
       <c r="P318" s="5"/>
     </row>
-    <row r="319" spans="1:16">
+    <row r="319" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A319" s="5" t="s">
         <v>297</v>
       </c>
@@ -17357,7 +17366,7 @@
       </c>
       <c r="P319" s="5"/>
     </row>
-    <row r="320" spans="1:16">
+    <row r="320" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A320" s="5" t="s">
         <v>298</v>
       </c>
@@ -17399,7 +17408,7 @@
       </c>
       <c r="P320" s="5"/>
     </row>
-    <row r="321" spans="1:16">
+    <row r="321" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A321" s="5" t="s">
         <v>299</v>
       </c>
@@ -17441,7 +17450,7 @@
       </c>
       <c r="P321" s="5"/>
     </row>
-    <row r="322" spans="1:16">
+    <row r="322" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A322" s="5" t="s">
         <v>300</v>
       </c>
@@ -17483,7 +17492,7 @@
       </c>
       <c r="P322" s="5"/>
     </row>
-    <row r="323" spans="1:16">
+    <row r="323" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A323" s="5" t="s">
         <v>301</v>
       </c>
@@ -17525,7 +17534,7 @@
       </c>
       <c r="P323" s="5"/>
     </row>
-    <row r="324" spans="1:16">
+    <row r="324" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A324" s="5" t="s">
         <v>302</v>
       </c>
@@ -17567,7 +17576,7 @@
       </c>
       <c r="P324" s="5"/>
     </row>
-    <row r="325" spans="1:16">
+    <row r="325" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A325" s="5" t="s">
         <v>303</v>
       </c>
@@ -17609,7 +17618,7 @@
       </c>
       <c r="P325" s="5"/>
     </row>
-    <row r="326" spans="1:16">
+    <row r="326" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A326" s="5" t="s">
         <v>304</v>
       </c>
@@ -17651,7 +17660,7 @@
       </c>
       <c r="P326" s="5"/>
     </row>
-    <row r="327" spans="1:16" hidden="1">
+    <row r="327" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A327" s="5" t="s">
         <v>305</v>
       </c>
@@ -17698,13 +17707,7 @@
       <c r="P327" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P327" xr:uid="{6F9B48B8-4818-484F-9B88-D707BC38F446}">
-    <filterColumn colId="14">
-      <filters>
-        <filter val="leonardo.cardona@uic.cu"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P327" xr:uid="{6F9B48B8-4818-484F-9B88-D707BC38F446}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G62:G76" xr:uid="{80CF0009-5974-4ECE-B407-1897D132CBDB}">

</xml_diff>